<commit_message>
Update store products via Admin Panel - 10/09/2026, 1:06:28 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="E96">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="F96">
         <v>65</v>
@@ -4395,10 +4395,10 @@
         <v/>
       </c>
       <c r="E97">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F97">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G97" t="str">
         <v>INSTOCK</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 15/09/2026, 7:58:02 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M278"/>
+  <dimension ref="A1:M277"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11758,10 +11758,10 @@
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>JW-68</v>
+        <v>JW-69</v>
       </c>
       <c r="B275" t="str">
-        <v>Necklace</v>
+        <v>Coral stone  necklace</v>
       </c>
       <c r="C275" t="str">
         <v>Jewellery</v>
@@ -11770,10 +11770,10 @@
         <v>Necklace</v>
       </c>
       <c r="E275">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="F275">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G275" t="str">
         <v>INSTOCK</v>
@@ -11782,10 +11782,10 @@
         <v/>
       </c>
       <c r="I275" t="str">
-        <v>d89f547f-6318-4301-abd2-ce3a5ba2b413.jpg</v>
+        <v>cf3f1c4c-56af-442c-b263-578fe3398ecb.jpg</v>
       </c>
       <c r="J275" t="str">
-        <v>f2ce700f-48b4-43f6-a6cb-61a36e8f7630.jpg</v>
+        <v>53aeff17-14ff-4155-b250-241f6154f0e9.jpg</v>
       </c>
       <c r="K275" t="str">
         <v/>
@@ -11799,10 +11799,10 @@
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>JW-69</v>
+        <v>JW-70</v>
       </c>
       <c r="B276" t="str">
-        <v>Coral stone  necklace</v>
+        <v>Lotus Necklace</v>
       </c>
       <c r="C276" t="str">
         <v>Jewellery</v>
@@ -11811,10 +11811,10 @@
         <v>Necklace</v>
       </c>
       <c r="E276">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="F276">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="G276" t="str">
         <v>INSTOCK</v>
@@ -11823,10 +11823,10 @@
         <v/>
       </c>
       <c r="I276" t="str">
-        <v>cf3f1c4c-56af-442c-b263-578fe3398ecb.jpg</v>
+        <v>9d2ebc31-ea0f-49ab-a8ce-cffcaccf16c3.jpg</v>
       </c>
       <c r="J276" t="str">
-        <v>53aeff17-14ff-4155-b250-241f6154f0e9.jpg</v>
+        <v>39ab9b5e-7afa-4301-b51a-281b998ae299.jpg</v>
       </c>
       <c r="K276" t="str">
         <v/>
@@ -11840,10 +11840,10 @@
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>JW-70</v>
+        <v>JW-71</v>
       </c>
       <c r="B277" t="str">
-        <v>Lotus Necklace</v>
+        <v>Necklace</v>
       </c>
       <c r="C277" t="str">
         <v>Jewellery</v>
@@ -11852,10 +11852,10 @@
         <v>Necklace</v>
       </c>
       <c r="E277">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F277">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G277" t="str">
         <v>INSTOCK</v>
@@ -11864,10 +11864,10 @@
         <v/>
       </c>
       <c r="I277" t="str">
-        <v>9d2ebc31-ea0f-49ab-a8ce-cffcaccf16c3.jpg</v>
+        <v>e96f5952-ad89-4eec-8f5b-741770b1d45a.jpg</v>
       </c>
       <c r="J277" t="str">
-        <v>39ab9b5e-7afa-4301-b51a-281b998ae299.jpg</v>
+        <v/>
       </c>
       <c r="K277" t="str">
         <v/>
@@ -11876,53 +11876,12 @@
         <v/>
       </c>
       <c r="M277" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="str">
-        <v>JW-71</v>
-      </c>
-      <c r="B278" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="C278" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D278" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="E278">
-        <v>26</v>
-      </c>
-      <c r="F278">
-        <v>32</v>
-      </c>
-      <c r="G278" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="H278" t="str">
-        <v/>
-      </c>
-      <c r="I278" t="str">
-        <v>e96f5952-ad89-4eec-8f5b-741770b1d45a.jpg</v>
-      </c>
-      <c r="J278" t="str">
-        <v/>
-      </c>
-      <c r="K278" t="str">
-        <v/>
-      </c>
-      <c r="L278" t="str">
-        <v/>
-      </c>
-      <c r="M278" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M278"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M277"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 16/09/2026, 5:39:28 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M277"/>
+  <dimension ref="A1:M280"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11879,9 +11879,132 @@
         <v>No</v>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>JW-72</v>
+      </c>
+      <c r="B278" t="str">
+        <v>CZ stone leaf pattern necklace set</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E278">
+        <v>46</v>
+      </c>
+      <c r="F278">
+        <v>55</v>
+      </c>
+      <c r="G278" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H278" t="str">
+        <v/>
+      </c>
+      <c r="I278" t="str">
+        <v>2b0491d5-9afb-4f6e-935c-2ca72d7f8192.jpg</v>
+      </c>
+      <c r="J278" t="str">
+        <v>76db279b-aa83-4ea8-a76a-84ece2744e40.jpg</v>
+      </c>
+      <c r="K278" t="str">
+        <v>3ddd9569-412d-4321-800f-e83a2d7592e4.jpg</v>
+      </c>
+      <c r="L278" t="str">
+        <v>Available in Mint green, Blush pink and Dark pink shades</v>
+      </c>
+      <c r="M278" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>JW-73</v>
+      </c>
+      <c r="B279" t="str">
+        <v>EXCLUSIVE TIKKA</v>
+      </c>
+      <c r="C279" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Chutti Matti</v>
+      </c>
+      <c r="E279">
+        <v>19</v>
+      </c>
+      <c r="F279">
+        <v>24</v>
+      </c>
+      <c r="G279" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H279" t="str">
+        <v/>
+      </c>
+      <c r="I279" t="str">
+        <v>63bccb34-ae0e-4108-aaf7-2012c9d40e99.jpg</v>
+      </c>
+      <c r="J279" t="str">
+        <v>cb6daf07-6218-4c03-adf4-cc98e995f7ab.jpg</v>
+      </c>
+      <c r="K279" t="str">
+        <v>1ea4917a-c783-4ada-9e21-a342c462d44d.jpg</v>
+      </c>
+      <c r="L279" t="str">
+        <v>Many beautiful varieties of tikkas are available in gold, silver, and rose-gold finishes.</v>
+      </c>
+      <c r="M279" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>JW-74</v>
+      </c>
+      <c r="B280" t="str">
+        <v>Premium CZ stone necklace set</v>
+      </c>
+      <c r="C280" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D280" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E280">
+        <v>46</v>
+      </c>
+      <c r="F280">
+        <v>54</v>
+      </c>
+      <c r="G280" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H280" t="str">
+        <v/>
+      </c>
+      <c r="I280" t="str">
+        <v>ee06fe9c-4b44-437f-8a09-5a25cf76966d.jpg</v>
+      </c>
+      <c r="J280" t="str">
+        <v/>
+      </c>
+      <c r="K280" t="str">
+        <v/>
+      </c>
+      <c r="L280" t="str">
+        <v>Few Pieces available</v>
+      </c>
+      <c r="M280" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M277"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M280"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 16/09/2026, 5:55:08 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M280"/>
+  <dimension ref="A1:M283"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12002,9 +12002,132 @@
         <v>No</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>JW-75</v>
+      </c>
+      <c r="B281" t="str">
+        <v>Kemp-Style Necklace set</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E281">
+        <v>46</v>
+      </c>
+      <c r="F281">
+        <v>52</v>
+      </c>
+      <c r="G281" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H281" t="str">
+        <v/>
+      </c>
+      <c r="I281" t="str">
+        <v>f7523ca8-eeae-4791-8ab8-9e95a4a62e17.jpg</v>
+      </c>
+      <c r="J281" t="str">
+        <v/>
+      </c>
+      <c r="K281" t="str">
+        <v/>
+      </c>
+      <c r="L281" t="str">
+        <v/>
+      </c>
+      <c r="M281" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>JW-76</v>
+      </c>
+      <c r="B282" t="str">
+        <v>Elegant gold-finish necklace set</v>
+      </c>
+      <c r="C282" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D282" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E282">
+        <v>36</v>
+      </c>
+      <c r="F282">
+        <v>44</v>
+      </c>
+      <c r="G282" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H282" t="str">
+        <v/>
+      </c>
+      <c r="I282" t="str">
+        <v>d74e8192-18ed-4ed9-a4db-a3d4e05d63a5.jpg</v>
+      </c>
+      <c r="J282" t="str">
+        <v>ebd05c37-c37a-4dae-a663-c704d9dcab54.jpg</v>
+      </c>
+      <c r="K282" t="str">
+        <v>adbe1261-4cbf-4b07-832f-abdd3f6239e8.jpg</v>
+      </c>
+      <c r="L282" t="str">
+        <v>Available 2 different shades.</v>
+      </c>
+      <c r="M282" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>JW-77</v>
+      </c>
+      <c r="B283" t="str">
+        <v>Elegant Floral CZ Necklace Set</v>
+      </c>
+      <c r="C283" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E283">
+        <v>42</v>
+      </c>
+      <c r="F283">
+        <v>49</v>
+      </c>
+      <c r="G283" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H283" t="str">
+        <v/>
+      </c>
+      <c r="I283" t="str">
+        <v>ac22057c-f2a9-4816-9580-22d549872b7b.jpg</v>
+      </c>
+      <c r="J283" t="str">
+        <v>04c3dcc3-f035-4f80-a93d-47449b479134.jpg</v>
+      </c>
+      <c r="K283" t="str">
+        <v/>
+      </c>
+      <c r="L283" t="str">
+        <v>Floral CZ Necklace Set ✨A graceful gold-toned necklace featuring delicate floral and leaf detailing, beautifully finished with sparkling clear CZ stones.</v>
+      </c>
+      <c r="M283" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M280"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M283"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 16/09/2026, 6:00:30 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -1427,7 +1427,7 @@
         <v>34</v>
       </c>
       <c r="G25" t="str">
-        <v>LIMITED STOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -5932,7 +5932,7 @@
         <v>14</v>
       </c>
       <c r="G134" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H134" t="str">
         <v/>
@@ -10833,7 +10833,7 @@
         <v>100</v>
       </c>
       <c r="G252" t="str">
-        <v>LIMITED STOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H252" t="str">
         <v/>
@@ -11155,10 +11155,10 @@
         <v/>
       </c>
       <c r="E260">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="F260">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G260" t="str">
         <v>LIMITED STOCK</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 16/09/2026, 6:01:15 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M283"/>
+  <dimension ref="A1:M282"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12004,10 +12004,10 @@
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>JW-75</v>
+        <v>JW-76</v>
       </c>
       <c r="B281" t="str">
-        <v>Kemp-Style Necklace set</v>
+        <v>Elegant gold-finish necklace set</v>
       </c>
       <c r="C281" t="str">
         <v>Jewellery</v>
@@ -12016,10 +12016,10 @@
         <v>Necklace</v>
       </c>
       <c r="E281">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="F281">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G281" t="str">
         <v>INSTOCK</v>
@@ -12028,16 +12028,16 @@
         <v/>
       </c>
       <c r="I281" t="str">
-        <v>f7523ca8-eeae-4791-8ab8-9e95a4a62e17.jpg</v>
+        <v>d74e8192-18ed-4ed9-a4db-a3d4e05d63a5.jpg</v>
       </c>
       <c r="J281" t="str">
-        <v/>
+        <v>ebd05c37-c37a-4dae-a663-c704d9dcab54.jpg</v>
       </c>
       <c r="K281" t="str">
-        <v/>
+        <v>adbe1261-4cbf-4b07-832f-abdd3f6239e8.jpg</v>
       </c>
       <c r="L281" t="str">
-        <v/>
+        <v>Available 2 different shades.</v>
       </c>
       <c r="M281" t="str">
         <v>No</v>
@@ -12045,10 +12045,10 @@
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>JW-76</v>
+        <v>JW-77</v>
       </c>
       <c r="B282" t="str">
-        <v>Elegant gold-finish necklace set</v>
+        <v>Elegant Floral CZ Necklace Set</v>
       </c>
       <c r="C282" t="str">
         <v>Jewellery</v>
@@ -12057,10 +12057,10 @@
         <v>Necklace</v>
       </c>
       <c r="E282">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F282">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="G282" t="str">
         <v>INSTOCK</v>
@@ -12069,65 +12069,24 @@
         <v/>
       </c>
       <c r="I282" t="str">
-        <v>d74e8192-18ed-4ed9-a4db-a3d4e05d63a5.jpg</v>
+        <v>ac22057c-f2a9-4816-9580-22d549872b7b.jpg</v>
       </c>
       <c r="J282" t="str">
-        <v>ebd05c37-c37a-4dae-a663-c704d9dcab54.jpg</v>
+        <v>04c3dcc3-f035-4f80-a93d-47449b479134.jpg</v>
       </c>
       <c r="K282" t="str">
-        <v>adbe1261-4cbf-4b07-832f-abdd3f6239e8.jpg</v>
+        <v/>
       </c>
       <c r="L282" t="str">
-        <v>Available 2 different shades.</v>
+        <v>Floral CZ Necklace Set ✨A graceful gold-toned necklace featuring delicate floral and leaf detailing, beautifully finished with sparkling clear CZ stones.</v>
       </c>
       <c r="M282" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="str">
-        <v>JW-77</v>
-      </c>
-      <c r="B283" t="str">
-        <v>Elegant Floral CZ Necklace Set</v>
-      </c>
-      <c r="C283" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D283" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="E283">
-        <v>42</v>
-      </c>
-      <c r="F283">
-        <v>49</v>
-      </c>
-      <c r="G283" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="H283" t="str">
-        <v/>
-      </c>
-      <c r="I283" t="str">
-        <v>ac22057c-f2a9-4816-9580-22d549872b7b.jpg</v>
-      </c>
-      <c r="J283" t="str">
-        <v>04c3dcc3-f035-4f80-a93d-47449b479134.jpg</v>
-      </c>
-      <c r="K283" t="str">
-        <v/>
-      </c>
-      <c r="L283" t="str">
-        <v>Floral CZ Necklace Set ✨A graceful gold-toned necklace featuring delicate floral and leaf detailing, beautifully finished with sparkling clear CZ stones.</v>
-      </c>
-      <c r="M283" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M283"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M282"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 16/09/2026, 6:18:30 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -2441,7 +2441,7 @@
         <v>Kids frocks</v>
       </c>
       <c r="C50" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D50" t="str">
         <v/>
@@ -2523,7 +2523,7 @@
         <v>FROCK</v>
       </c>
       <c r="C52" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D52" t="str">
         <v/>
@@ -2688,7 +2688,7 @@
         <v>Necklace</v>
       </c>
       <c r="C56" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D56" t="str">
         <v/>
@@ -2975,10 +2975,10 @@
         <v>Jewellery</v>
       </c>
       <c r="C63" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D63" t="str">
-        <v/>
+        <v>Bangles</v>
       </c>
       <c r="E63">
         <v>15</v>
@@ -3140,7 +3140,7 @@
         <v>Kids frocks</v>
       </c>
       <c r="C67" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D67" t="str">
         <v/>
@@ -3183,13 +3183,13 @@
         <v>Kids frocks</v>
       </c>
       <c r="C68" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D68" t="str">
         <v/>
       </c>
       <c r="E68">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F68">
         <v>30</v>
@@ -3389,10 +3389,10 @@
         <v>Premium double layer</v>
       </c>
       <c r="C73" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D73" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E73">
         <v>39</v>
@@ -4223,13 +4223,13 @@
         <v>Kids pattupavada</v>
       </c>
       <c r="C93" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D93" t="str">
         <v/>
       </c>
       <c r="E93">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F93">
         <v>58</v>
@@ -5715,10 +5715,10 @@
         <v>NGAPADAM  necklace</v>
       </c>
       <c r="C129" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D129" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E129">
         <v>29</v>
@@ -6166,10 +6166,10 @@
         <v>Casual wear</v>
       </c>
       <c r="C140" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D140" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E140">
         <v>12</v>
@@ -6617,10 +6617,10 @@
         <v>Premium   stone necklace</v>
       </c>
       <c r="C151" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D151" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E151">
         <v>33</v>
@@ -6659,10 +6659,10 @@
         <v>Jhumka</v>
       </c>
       <c r="C152" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D152" t="str">
-        <v/>
+        <v>Earring</v>
       </c>
       <c r="E152">
         <v>13</v>
@@ -6701,10 +6701,10 @@
         <v>Casual earrings</v>
       </c>
       <c r="C153" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D153" t="str">
-        <v/>
+        <v>Earring</v>
       </c>
       <c r="E153">
         <v>12</v>
@@ -7603,7 +7603,7 @@
         <v>Invisible necklace</v>
       </c>
       <c r="C175" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D175" t="str">
         <v/>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/09/2026, 4:41:06 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -1591,7 +1591,7 @@
         <v>14</v>
       </c>
       <c r="G29" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -2453,7 +2453,7 @@
         <v>23.69</v>
       </c>
       <c r="G50" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -3237,7 +3237,7 @@
         <v>32</v>
       </c>
       <c r="G69" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -11530,7 +11530,7 @@
         <v>65</v>
       </c>
       <c r="G269" t="str">
-        <v>LIMITED STOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H269" t="str">
         <v>38</v>

</xml_diff>